<commit_message>
UK daily ratings for 2026-05-04
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-04.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-04.xlsx
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Tricky Jenny</t>
+          <t>Dees Star (IRE)</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Dees Star (IRE)</t>
+          <t>Devon Angel</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Devon Angel</t>
+          <t>Tricky Jenny</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Marty Hopkirk (IRE)</t>
+          <t>Desert Cop</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J26" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="K26" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2008,17 +2008,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Desert Cop</t>
+          <t>Marty Hopkirk (IRE)</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K27" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -3916,17 +3916,17 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Lady Of Clover (IRE)</t>
+          <t>Henfield</t>
         </is>
       </c>
       <c r="I59" t="n">
         <v>3</v>
       </c>
       <c r="J59" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K59" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
@@ -3972,17 +3972,17 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Henfield</t>
+          <t>Lady Of Clover (IRE)</t>
         </is>
       </c>
       <c r="I60" t="n">
         <v>3</v>
       </c>
       <c r="J60" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K60" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="n">
@@ -7592,17 +7592,17 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>The Pug (IRE)</t>
+          <t>Daring Leader (IRE)</t>
         </is>
       </c>
       <c r="I121" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J121" t="n">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="K121" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="n">
@@ -7648,17 +7648,17 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Daring Leader (IRE)</t>
+          <t>The Pug (IRE)</t>
         </is>
       </c>
       <c r="I122" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J122" t="n">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="K122" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
@@ -15852,26 +15852,26 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Thats Random</t>
+          <t>Bundok</t>
         </is>
       </c>
       <c r="I263" t="n">
         <v>3</v>
       </c>
       <c r="J263" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K263" t="n">
         <v>0</v>
       </c>
       <c r="L263" t="n">
-        <v>8.15</v>
+        <v>6.65</v>
       </c>
       <c r="M263" t="n">
         <v>72.56</v>
       </c>
       <c r="N263" t="n">
-        <v>55.7</v>
+        <v>55.6</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -15879,7 +15879,7 @@
         </is>
       </c>
       <c r="P263" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="264">
@@ -15912,14 +15912,14 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Bundok</t>
+          <t>Thats Random</t>
         </is>
       </c>
       <c r="I264" t="n">
         <v>3</v>
       </c>
       <c r="J264" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K264" t="n">
         <v>0</v>
@@ -15931,7 +15931,7 @@
         <v>72.56</v>
       </c>
       <c r="N264" t="n">
-        <v>51.4</v>
+        <v>55.7</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -15939,7 +15939,7 @@
         </is>
       </c>
       <c r="P264" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265">
@@ -20436,14 +20436,14 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>Turret (IRE)</t>
+          <t>Symphonys Song</t>
         </is>
       </c>
       <c r="I340" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J340" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K340" t="n">
         <v>0</v>
@@ -20492,7 +20492,7 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>Windbreaker</t>
+          <t>Turret (IRE)</t>
         </is>
       </c>
       <c r="I341" t="n">
@@ -20548,14 +20548,14 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>Symphonys Song</t>
+          <t>Windbreaker</t>
         </is>
       </c>
       <c r="I342" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J342" t="n">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="K342" t="n">
         <v>0</v>
@@ -21262,17 +21262,17 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>Tinsel</t>
+          <t>La Peregrina</t>
         </is>
       </c>
       <c r="I354" t="n">
         <v>3</v>
       </c>
       <c r="J354" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K354" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L354" t="inlineStr"/>
       <c r="M354" t="n">
@@ -21318,17 +21318,17 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>La Peregrina</t>
+          <t>Tinsel</t>
         </is>
       </c>
       <c r="I355" t="n">
         <v>3</v>
       </c>
       <c r="J355" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K355" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L355" t="inlineStr"/>
       <c r="M355" t="n">
@@ -23698,17 +23698,17 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>Man From Havana</t>
+          <t>Blackwaterfoot (USA)</t>
         </is>
       </c>
       <c r="I395" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J395" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K395" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="L395" t="inlineStr"/>
       <c r="M395" t="n">
@@ -23754,17 +23754,17 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>Blackwaterfoot (USA)</t>
+          <t>Man From Havana</t>
         </is>
       </c>
       <c r="I396" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J396" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K396" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="L396" t="inlineStr"/>
       <c r="M396" t="n">

</xml_diff>